<commit_message>
Leads: 2026-10-11 06:10 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,66 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Llagua Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>llaguaroofing.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://llaguaroofing.com/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Central Texas</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>info@llaguaroofing.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(737) 808-2324</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Austin TX</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>roof repair company Austin TX</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 06:13 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Plumb Texan</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>plumbtexan.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://plumbtexan.com/round-rock-plumber/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Central Texas</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>aaron@plumbtexan.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(512) 966-0624</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Round Rock TX</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>plumber Round Rock TX</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 14:53 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,62 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MRJ Plumbing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>mrjplumbing.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.mrjplumbing.com/service-areas/asheville-nc</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>marcel@mrjplumbing.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(828) 222-3903</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Asheville NC</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>plumbing company Asheville NC</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 14:57 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -704,7 +704,6 @@
           <t>https://www.mrjplumbing.com/service-areas/asheville-nc</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>marcel@mrjplumbing.com</t>
@@ -734,6 +733,66 @@
         </is>
       </c>
       <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Plumber Tulsa, OK | Golden Rule Plumbing and Drains</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>tulsagoldenrule.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://tulsagoldenrule.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Learn More</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>info@tulsagoldenrule.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>9188079569</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Tulsa OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>plumber Tulsa OK</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-11 15:05 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,62 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AC Sales</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ac-sales.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.ac-sales.com/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>jlege@ac-sales.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>337.234.2345</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Lafayette LA</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>heat pump installation Lafayette LA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 15:06 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -819,7 +819,6 @@
           <t>https://www.ac-sales.com/heat-pump-installation</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>jlege@ac-sales.com</t>
@@ -849,6 +848,62 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bureau of Sanitary and Stormwater Sewers</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pd.cmvny.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://pd.cmvny.com/910/Bureau-of-Sanitary-and-Stormwater-Sewers</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>amontero@cmvny.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>914-665-2465</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>84</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>sewer repair Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-11 15:08 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -874,7 +874,6 @@
           <t>https://pd.cmvny.com/910/Bureau-of-Sanitary-and-Stormwater-Sewers</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>amontero@cmvny.com</t>
@@ -904,6 +903,66 @@
         </is>
       </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Right There Plumbing, LLC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>rightthereplumbing.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.rightthereplumbing.com/plumber-lexington-ky/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Your Trusted</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>rightthereplumbing23@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(859) 481-5654</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>emergency plumber Lexington KY</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-11 15:09 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -968,6 +968,66 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>John Hirt Construction</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>jhirtconstruction.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.jhirtconstruction.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Company Built</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>austinb@jhirtconstruction.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(608) 608-1046</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Madison WI</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>86</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roofing contractor Madison WI</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 20:05 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1028,6 +1028,66 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tecta America</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>tectaamerica.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.tectaamerica.com/location/bandlsheetmetalandroofing/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>David Lee</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@tectaamerica.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(812) 332-4309</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Bloomington IN</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>96</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Bloomington IN</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 20:06 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1088,6 +1088,62 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Strive HVAC &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>strivehvac.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.strivehvac.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@strivehvac.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(832) 275-6615</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Houston TX</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>HVAC contractor Houston TX</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 20:08 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1109,7 +1109,6 @@
           <t>https://www.strivehvac.com/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>info@strivehvac.com</t>
@@ -1139,6 +1138,66 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Signature Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>signatureairusa.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://signatureairusa.com/service-areas/pompano-beach</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Heat Pump</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>jcmcoldair@aol.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(954) 457-4560</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Pompano Beach FL</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>air conditioning repair Pompano Beach FL</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-11 20:11 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1203,6 +1203,62 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Professional Plumbers in Hialeah, FL | Quality Service</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>hialeahplumbing.net</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.hialeahplumbing.net/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>mymail@mailservice.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>555-555-5555</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Hialeah FL</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>plumber Hialeah FL</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 20:18 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1224,7 +1224,6 @@
           <t>https://www.hialeahplumbing.net/</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>mymail@mailservice.com</t>
@@ -1254,6 +1253,126 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Riverside Plumbing Pros</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>plumbingriversidepro.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://plumbingriversidepro.com/water-heater-installation-repair/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Riverside Plumbing</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>dispatch@plumbingriversidepro.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(831) 290-4327</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Riverside CA</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>water heater repair Riverside CA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Arthur's Roofing</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>arthursroofing.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://arthursroofing.com/services/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Triad Word</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>office@arthursroofing.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(336) 565-5585</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Greensboro NC</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Greensboro NC</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-11 23:25 UTC (cycle 139)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1378,6 +1378,126 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ProShield Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>proshieldroofing.org</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://proshieldroofing.org/roofing-services-fishers-in/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Homeowner Resources</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>office@proshieldroofing.org</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>317-764-9811</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Fishers IN</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>roof repair company Fishers IN</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Fishers IN Roofing Company | Roof Repair &amp; Replacement | Martinez Roofing &amp; More</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>martinezroofingmore.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.martinezroofingmore.com/roofing/fishers</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Say Don</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>jrhall2130@gmail.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(317) 822-1846</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Fishers IN</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>90</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>roof repair company Fishers IN</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 23:28 UTC (cycle 141)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1498,6 +1498,62 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>sky-bright Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>skybrightroofing.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.skybrightroofing.com/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Oliver Hartman</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>support@webador.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Portland OR</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>76</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Portland OR</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 23:31 UTC (cycle 143)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1529,7 +1529,6 @@
           <t>support@webador.com</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Portland OR</t>
@@ -1549,6 +1548,66 @@
         </is>
       </c>
       <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>J &amp; K Roofing</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>jkroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://jkroofinginc.com/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Building Roof</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>julio@jkroofinginc.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(954) 961-9879</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Hollywood FL</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>98</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>residential roofing company Hollywood FL</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-11 23:50 UTC (cycle 156)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1613,6 +1613,62 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Roofing Contractor | Five Star Roofing Corp | Hialeah, FL</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>fivestar-roofing.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.fivestar-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>maria@fivestar-roofing.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(305) 231-7195</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Hialeah FL</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>90</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>roofing contractor Hialeah FL</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 23:53 UTC (cycle 158)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1634,7 +1634,6 @@
           <t>https://www.fivestar-roofing.com/</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>maria@fivestar-roofing.com</t>
@@ -1664,6 +1663,66 @@
         </is>
       </c>
       <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Tri Express Plumbing</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>triexpressplumbing.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://triexpressplumbing.com/emergency-plumber-chula-vista/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>info@triexpressplumbing.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>(619) 843-6692</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Chula Vista CA</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>90</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>emergency plumber Chula Vista CA</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>2026-10-11</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-11 23:54 UTC (cycle 159)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1728,6 +1728,66 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Creatum Roofing and Repair</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>creatumconstruction.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.creatumconstruction.com/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Creatum Roofing</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>creatumroofingandrepair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(406)404-8400</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Missoula MT</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>90</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>roof replacement Missoula MT</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 23:56 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1788,6 +1788,66 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ProLine Plumbing OKC</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>prolineplumbingokc.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://prolineplumbingokc.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Cleaning Clogged</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>brandon@prolineplumbingokc.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(405) 517-8640</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Oklahoma City OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>90</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>plumbing company Oklahoma City OK</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 23:58 UTC (cycle 161)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1848,6 +1848,66 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Dallas Roofings</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>dallasroofings.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.dallasroofings.com/</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Dallas Roofings</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>info@dallasroofings.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(945) 319-8441</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Dallas TX</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>roof repair company Dallas TX</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-11 23:59 UTC (cycle 162)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-11.xlsx
+++ b/output/leads_2026-10-11.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1908,6 +1908,66 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Emergency Plumber Chattanooga, TN | Chattanooga Expert Plumber</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>chattanoogaexpertplumber.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://chattanoogaexpertplumber.com/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Chattanooga Expert</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>contact@chattanoogaexpertplumber.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>(423) 810-4269</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>90</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>emergency plumber Chattanooga TN</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>